<commit_message>
parameters not completed yet
</commit_message>
<xml_diff>
--- a/data/PREBAS_parameters.xlsx
+++ b/data/PREBAS_parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="pPRELES" sheetId="1" state="visible" r:id="rId3"/>
@@ -15,6 +15,7 @@
     <sheet name="pClearcut" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="pAWEN" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="pHcM" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="pPeattp" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,8 +26,62 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>tc={02ED04FC-0899-419C-B1CD-2DBC115BE9A6}</author>
+  </authors>
+  <commentList>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Soilmodel = 1 - parameters are required for all versions
+Soilmodel  = 2 - parameters are required for peatland version only</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>tc={16BD7AB2-0687-4CF3-B9E5-7089840607E3}</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Soilmodel = 1 - parameters are required for all versions
+Soilmodel  = 2 - parameters are required for peatland version only</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="246">
   <si>
     <t xml:space="preserve">pPRELESnames</t>
   </si>
@@ -55,21 +110,87 @@
     <t xml:space="preserve">Catalonia</t>
   </si>
   <si>
+    <t xml:space="preserve">parClass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soilmodel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">definition</t>
+  </si>
+  <si>
     <t xml:space="preserve">soildepth</t>
   </si>
   <si>
+    <t xml:space="preserve">Site_par</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Effective field capacity</t>
   </si>
   <si>
+    <t xml:space="preserve">unitless</t>
+  </si>
+  <si>
     <t xml:space="preserve">Permanent wilting point</t>
   </si>
   <si>
     <t xml:space="preserve">Drainage delay</t>
   </si>
   <si>
+    <t xml:space="preserve">d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">topdepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depth of top layer which is source for evaporation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orgthres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">threshold parameter for top layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oveflow storage for top layer, usually 1 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ditchDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dpth of ditches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ditchDist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">distance between ditches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peatDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt; ditchDepth, depth to which soil water is calculated, differs from soil depth which is rooting depth</t>
+  </si>
+  <si>
     <t xml:space="preserve">LUE</t>
   </si>
   <si>
+    <t xml:space="preserve">GPP_par</t>
+  </si>
+  <si>
     <t xml:space="preserve">tauGPP</t>
   </si>
   <si>
@@ -94,9 +215,18 @@
     <t xml:space="preserve"> xCO2</t>
   </si>
   <si>
+    <t xml:space="preserve">soils</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter for smooth soil water response model</t>
+  </si>
+  <si>
     <t xml:space="preserve">transpiration efficiency </t>
   </si>
   <si>
+    <t xml:space="preserve">ET_par</t>
+  </si>
+  <si>
     <t xml:space="preserve">kappaET</t>
   </si>
   <si>
@@ -112,6 +242,9 @@
     <t xml:space="preserve">Metlcoeff</t>
   </si>
   <si>
+    <t xml:space="preserve">SnowRain_par</t>
+  </si>
+  <si>
     <t xml:space="preserve"> I_0 </t>
   </si>
   <si>
@@ -127,6 +260,9 @@
     <t xml:space="preserve"> Swinit</t>
   </si>
   <si>
+    <t xml:space="preserve">Init_par</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cwinit</t>
   </si>
   <si>
@@ -136,6 +272,18 @@
     <t xml:space="preserve">Sinit</t>
   </si>
   <si>
+    <t xml:space="preserve">Stinit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">initial water level in top layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wlinit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">initial water table depth, mm, needs to be synchronised with water storage SW, to be consistent with SWTable</t>
+  </si>
+  <si>
     <t xml:space="preserve"> t0 </t>
   </si>
   <si>
@@ -560,16 +708,128 @@
   </si>
   <si>
     <t xml:space="preserve">NA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peattype_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peattype_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thetaS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genuchten_par</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm/mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">porosity </t>
+  </si>
+  <si>
+    <t xml:space="preserve">from 0.1 m to peatDepth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thetaR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">residual water content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">air entry suction </t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pore size distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thetaST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">porosity of peat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">from top to 0.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thetaRT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alphaT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saturated soil hydraulic conductivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">distribution within 0 and 2 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks(12)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00E+00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -591,6 +851,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -658,7 +924,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -911,7 +1177,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr defaultColWidth="8.3828125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.27"/>
@@ -946,10 +1212,22 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>413</v>
@@ -975,10 +1253,19 @@
       <c r="I2" s="1" t="n">
         <v>760.148203499524</v>
       </c>
+      <c r="J2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.45</v>
@@ -1004,10 +1291,19 @@
       <c r="I3" s="1" t="n">
         <v>0.45</v>
       </c>
+      <c r="J3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.118</v>
@@ -1033,10 +1329,19 @@
       <c r="I4" s="1" t="n">
         <v>0.118</v>
       </c>
+      <c r="J4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>3</v>
@@ -1062,759 +1367,1293 @@
       <c r="I5" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>0.7457</v>
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1.004588094</v>
+        <v>-999</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.820124449</v>
+        <v>-999</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.710401999</v>
+        <v>-999</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.723914797</v>
+        <v>-999</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.783982507431094</v>
+        <v>-999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.6928756</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0.753635191601492</v>
+        <v>-999</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>10.93</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>2.187171797</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>5.650375927</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>15.53840697</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>12.58078446</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>5.40766132920764</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>10.96842</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>11.0637921074664</v>
+      <c r="K7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>-3.063</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>-9.937886741</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>-3.19169985</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>3.43708684</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>2.987248049</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>-8.72893919193914</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>-3.932096</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>-1.82462599794009</v>
+      <c r="M8" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>17.72</v>
+        <v>27</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>23.33402032</v>
+        <v>-999</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>17.45828968</v>
+        <v>-999</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>10.75103013</v>
+        <v>-999</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>12.36089352</v>
+        <v>-999</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>26.7630451523391</v>
+        <v>-999</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>19.99568</v>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>18.5698913508732</v>
+        <v>-999</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>-0.1027</v>
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>30</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.078699766</v>
+        <v>-999</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>-0.158842341</v>
+        <v>-999</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.325620279</v>
+        <v>-999</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-0.214970139</v>
+        <v>-999</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>-0.119582403900148</v>
+        <v>-999</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>-0.1016437</v>
-      </c>
-      <c r="I10" s="1" t="n">
-        <v>-0.138440272468953</v>
+        <v>-999</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>0.03673</v>
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>2000</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.05678157</v>
+        <v>-999</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.033324665</v>
+        <v>-999</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.012187446</v>
+        <v>-999</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.019216213</v>
+        <v>-999</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.034855279860314</v>
+        <v>-999</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.03541814</v>
-      </c>
-      <c r="I11" s="1" t="n">
-        <v>0.0974307211287034</v>
+        <v>-999</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.7779</v>
+        <v>0.7457</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.43569651</v>
+        <v>1.004588094</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.650491581</v>
+        <v>0.820124449</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.365334323</v>
+        <v>0.710401999</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.257387576</v>
+        <v>0.723914797</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.791474635592007</v>
+        <v>0.783982507431094</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.3085413</v>
+        <v>0.6928756</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>0.485549685871757</v>
+        <v>0.753635191601492</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>2000</v>
+        <v>10.93</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2000</v>
+        <v>2.187171797</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2000</v>
+        <v>5.650375927</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2000</v>
+        <v>15.53840697</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>2000</v>
+        <v>12.58078446</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>2000</v>
+        <v>5.40766132920764</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>2000</v>
+        <v>10.96842</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>2000</v>
+        <v>11.0637921074664</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.4</v>
+        <v>-3.063</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.4</v>
+        <v>-9.937886741</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.4</v>
+        <v>-3.19169985</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.4</v>
+        <v>3.43708684</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.4</v>
+        <v>2.987248049</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.4</v>
+        <v>-8.72893919193914</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0.4</v>
+        <v>-3.932096</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0.4</v>
+        <v>-1.82462599794009</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.2715</v>
+        <v>17.72</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.216867322</v>
+        <v>23.33402032</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.119428078</v>
+        <v>17.45828968</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.230181468</v>
+        <v>10.75103013</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.279942541</v>
+        <v>12.36089352</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.230837102742928</v>
+        <v>26.7630451523391</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.2672472</v>
+        <v>19.99568</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>0.703098488490787</v>
+        <v>18.5698913508732</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>0.8351</v>
+        <v>-0.1027</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.886165542</v>
+        <v>-0.078699766</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.899640533</v>
+        <v>-0.158842341</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.712259738</v>
+        <v>-0.325620279</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.678182346</v>
+        <v>-0.214970139</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.756951384503756</v>
+        <v>-0.119582403900148</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0.895047</v>
+        <v>-0.1016437</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>0.830537812426035</v>
+        <v>-0.138440272468953</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0.07348</v>
+        <v>0.03673</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.076537373</v>
+        <v>0.05678157</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.163152905</v>
+        <v>0.033324665</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.102780391</v>
+        <v>0.012187446</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.036205559</v>
+        <v>0.019216213</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.098397649465536</v>
+        <v>0.034855279860314</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0.09091077</v>
+        <v>0.03541814</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>0.0177089959735055</v>
+        <v>0.0974307211287034</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>0.9996</v>
+        <v>0.7779</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.250944646</v>
+        <v>0.43569651</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.999200597</v>
+        <v>0.650491581</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.999244122</v>
+        <v>0.365334323</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.000912058</v>
+        <v>0.257387576</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.999515961301202</v>
+        <v>0.791474635592007</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0.8098139</v>
+        <v>0.3085413</v>
       </c>
       <c r="I18" s="1" t="n">
-        <v>0.602602442065657</v>
+        <v>0.485549685871757</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>0.4428</v>
+        <v>2000</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.484834199</v>
+        <v>2000</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.623269245</v>
+        <v>2000</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.622317794</v>
+        <v>2000</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.976139923</v>
+        <v>2000</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.195616291162648</v>
+        <v>2000</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>0.004138743</v>
+        <v>2000</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>0.461894616762674</v>
+        <v>2000</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0.33</v>
+        <v>-15</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.33</v>
+        <v>-999</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.33</v>
+        <v>-999</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.33</v>
+        <v>-999</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.33</v>
+        <v>-999</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.33</v>
+        <v>-999</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="I21" s="1" t="n">
-        <v>0.33</v>
+        <v>-999</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>4.970496</v>
+        <v>0.2715</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.992544622</v>
+        <v>0.216867322</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>4.35800751</v>
+        <v>0.119428078</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>5.201515182</v>
+        <v>0.230181468</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>4.970496</v>
+        <v>0.279942541</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>6.16</v>
+        <v>0.230837102742928</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>5.847971</v>
+        <v>0.2672472</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>3.16582976025463</v>
+        <v>0.703098488490787</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0</v>
+        <v>0.8351</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0</v>
+        <v>0.886165542</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>0.899640533</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>0.712259738</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>0.678182346</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>0.756951384503756</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>0.895047</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>0</v>
+        <v>0.830537812426035</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0</v>
+        <v>0.07348</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>0.076537373</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>0.163152905</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>0.102780391</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>0.036205559</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0</v>
+        <v>0.098397649465536</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0</v>
+        <v>0.09091077</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>0</v>
+        <v>0.0177089959735055</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>160</v>
+        <v>0.9996</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>160</v>
+        <v>0.250944646</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>200</v>
+        <v>0.999200597</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>200</v>
+        <v>0.999244122</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>200</v>
+        <v>0.000912058</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>200</v>
+        <v>0.999515961301202</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>160</v>
+        <v>0.8098139</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>160</v>
+        <v>0.602602442065657</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0</v>
+        <v>0.4428</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
+        <v>2.484834199</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>0.623269245</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>0.622317794</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>0.976139923</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>0.195616291162648</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>0</v>
+        <v>0.004138743</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>0</v>
+        <v>0.461894616762674</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>0</v>
+        <v>1.2</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>20</v>
+        <v>0.33</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>20</v>
+        <v>0.33</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>-7.9532</v>
+        <v>0.33</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1.8857</v>
+        <v>0.33</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>20</v>
+        <v>0.33</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>20</v>
+        <v>0.33</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>-999</v>
+        <v>4.970496</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>-999</v>
+        <v>0.992544622</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-999</v>
+        <v>4.35800751</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-999</v>
+        <v>5.201515182</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-999</v>
+        <v>4.970496</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>-999</v>
+        <v>6.16</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>-999</v>
+        <v>5.847971</v>
       </c>
       <c r="I29" s="1" t="n">
-        <v>-999</v>
+        <v>3.16582976025463</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>-999</v>
+        <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>-999</v>
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="B31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="I32" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>-7.9532</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>1.8857</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I35" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="C36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="D36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="D31" s="2" t="n">
+      <c r="E36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="F36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="H36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="I36" s="2" t="n">
         <v>-999</v>
       </c>
-      <c r="I31" s="1" t="n">
+      <c r="J36" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="C37" s="2" t="n">
         <v>-999</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I38" s="1" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I39" s="1" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I40" s="1" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1825,6 +2664,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1844,19 +2684,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1864,16 +2704,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,16 +2721,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,16 +2738,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1915,16 +2755,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1932,16 +2772,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1949,16 +2789,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1966,16 +2806,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>66</v>
+        <v>97</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>68</v>
+        <v>99</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1983,16 +2823,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2000,16 +2840,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2017,16 +2857,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,16 +2874,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>80</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2051,16 +2891,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2068,16 +2908,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2085,16 +2925,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2102,16 +2942,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2119,16 +2959,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2136,16 +2976,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2153,16 +2993,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2170,16 +3010,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>100</v>
+        <v>131</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2187,16 +3027,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2204,16 +3044,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2221,16 +3061,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2258,78 +3098,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>115</v>
+        <v>146</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>119</v>
+        <v>150</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0.22406007</v>
@@ -2400,7 +3240,7 @@
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>195.1657175</v>
@@ -2471,7 +3311,7 @@
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>20.00788979</v>
@@ -2542,7 +3382,7 @@
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>125</v>
+        <v>156</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.2500324</v>
@@ -2613,7 +3453,7 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>126</v>
+        <v>157</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>3.90739583</v>
@@ -2684,7 +3524,7 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.9077799</v>
@@ -2755,7 +3595,7 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.29990356</v>
@@ -2826,7 +3666,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>129</v>
+        <v>160</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.4</v>
@@ -2897,7 +3737,7 @@
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.5</v>
@@ -2968,7 +3808,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>131</v>
+        <v>162</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.03002172</v>
@@ -3039,7 +3879,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1.79017546</v>
@@ -3110,7 +3950,7 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>133</v>
+        <v>164</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.2869018</v>
@@ -3181,7 +4021,7 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>134</v>
+        <v>165</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.39976573</v>
@@ -3252,7 +4092,7 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>135</v>
+        <v>166</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.3800673</v>
@@ -3323,7 +4163,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>136</v>
+        <v>167</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>180.2348166</v>
@@ -3394,7 +4234,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>137</v>
+        <v>168</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.01052194</v>
@@ -3465,7 +4305,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>138</v>
+        <v>169</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>855.0095222</v>
@@ -3536,7 +4376,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>139</v>
+        <v>170</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.97559558</v>
@@ -3607,7 +4447,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>140</v>
+        <v>171</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.8</v>
@@ -3678,7 +4518,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>141</v>
+        <v>172</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.687</v>
@@ -3749,7 +4589,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>142</v>
+        <v>173</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.4</v>
@@ -3820,7 +4660,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>143</v>
+        <v>174</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.44</v>
@@ -3891,7 +4731,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>144</v>
+        <v>175</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0.47</v>
@@ -3962,7 +4802,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>0.64</v>
@@ -4033,7 +4873,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>0.84</v>
@@ -4104,7 +4944,7 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
@@ -4175,7 +5015,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
@@ -4246,7 +5086,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>149</v>
+        <v>180</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
@@ -4317,7 +5157,7 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>150</v>
+        <v>181</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1.4</v>
@@ -4388,7 +5228,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1250</v>
@@ -4459,7 +5299,7 @@
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>0</v>
@@ -4530,7 +5370,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>33</v>
@@ -4601,7 +5441,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>154</v>
+        <v>185</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>0.03</v>
@@ -4672,7 +5512,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>0.000669</v>
@@ -4743,7 +5583,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>-2.653</v>
@@ -4814,7 +5654,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>0.055</v>
@@ -4885,7 +5725,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>-0.03</v>
@@ -4956,7 +5796,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>159</v>
+        <v>190</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>0.07</v>
@@ -5027,7 +5867,7 @@
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>160</v>
+        <v>191</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>20.00788979</v>
@@ -5098,7 +5938,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>161</v>
+        <v>192</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>0</v>
@@ -5169,7 +6009,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>1</v>
@@ -5240,7 +6080,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>2.7801</v>
@@ -5311,7 +6151,7 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>0.9395</v>
@@ -5382,7 +6222,7 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1.191</v>
@@ -5453,7 +6293,7 @@
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
@@ -5524,7 +6364,7 @@
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>2.5</v>
@@ -5595,7 +6435,7 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>0.8</v>
@@ -5666,7 +6506,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>9.999</v>
@@ -5737,7 +6577,7 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>0.66</v>
@@ -5808,7 +6648,7 @@
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>-9999</v>
@@ -5879,7 +6719,7 @@
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>-9999</v>
@@ -5950,7 +6790,7 @@
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>-9999</v>
@@ -6021,7 +6861,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>-9999</v>
@@ -6111,16 +6951,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -6144,7 +6984,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0.2499834</v>
@@ -6177,7 +7017,7 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>208.3953</v>
@@ -6210,7 +7050,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>21.48298</v>
@@ -6243,7 +7083,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>125</v>
+        <v>156</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.3132079</v>
@@ -6276,7 +7116,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>126</v>
+        <v>157</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>3.850065</v>
@@ -6309,7 +7149,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.8716194</v>
@@ -6342,7 +7182,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.2994706</v>
@@ -6375,7 +7215,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>129</v>
+        <v>160</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.2154444</v>
@@ -6408,7 +7248,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.2014719</v>
@@ -6441,7 +7281,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>131</v>
+        <v>162</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.03937977</v>
@@ -6474,7 +7314,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1.9067</v>
@@ -6507,7 +7347,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>133</v>
+        <v>164</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.2866436</v>
@@ -6540,7 +7380,7 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>134</v>
+        <v>165</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.3996897</v>
@@ -6573,7 +7413,7 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>135</v>
+        <v>166</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.3017396</v>
@@ -6606,7 +7446,7 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>136</v>
+        <v>167</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>244</v>
@@ -6639,7 +7479,7 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>137</v>
+        <v>168</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0</v>
@@ -6672,7 +7512,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>138</v>
+        <v>169</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>668.7807</v>
@@ -6705,7 +7545,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>139</v>
+        <v>170</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.4000692</v>
@@ -6738,7 +7578,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>140</v>
+        <v>171</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.8</v>
@@ -6771,7 +7611,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>141</v>
+        <v>172</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.687</v>
@@ -6804,7 +7644,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>142</v>
+        <v>173</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.3755139</v>
@@ -6837,7 +7677,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>143</v>
+        <v>174</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.3864066</v>
@@ -6870,7 +7710,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>144</v>
+        <v>175</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0.5608545</v>
@@ -6903,7 +7743,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>0.5369738</v>
@@ -6936,7 +7776,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>0.7315046</v>
@@ -6969,7 +7809,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
@@ -7002,7 +7842,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
@@ -7035,7 +7875,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>149</v>
+        <v>180</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
@@ -7068,7 +7908,7 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>150</v>
+        <v>181</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1.4</v>
@@ -7101,7 +7941,7 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1250</v>
@@ -7134,7 +7974,7 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>0</v>
@@ -7167,7 +8007,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>33</v>
@@ -7200,7 +8040,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>154</v>
+        <v>185</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>0.03</v>
@@ -7233,7 +8073,7 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>0.000669</v>
@@ -7266,7 +8106,7 @@
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>-2.653</v>
@@ -7299,7 +8139,7 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>0.055</v>
@@ -7332,7 +8172,7 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>-0.03</v>
@@ -7365,7 +8205,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>159</v>
+        <v>190</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>0.076518</v>
@@ -7398,7 +8238,7 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>160</v>
+        <v>191</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>20.00789</v>
@@ -7431,7 +8271,7 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>161</v>
+        <v>192</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>0</v>
@@ -7464,7 +8304,7 @@
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>1</v>
@@ -7497,7 +8337,7 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>2.7801</v>
@@ -7530,7 +8370,7 @@
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>0.9395</v>
@@ -7563,7 +8403,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1.191</v>
@@ -7596,7 +8436,7 @@
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
@@ -7629,7 +8469,7 @@
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>2.5</v>
@@ -7662,7 +8502,7 @@
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>0.8</v>
@@ -7695,7 +8535,7 @@
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>9.999</v>
@@ -7728,7 +8568,7 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>0.66</v>
@@ -7761,7 +8601,7 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>-9999</v>
@@ -7794,7 +8634,7 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>-9999</v>
@@ -7827,7 +8667,7 @@
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>-9999</v>
@@ -7860,7 +8700,7 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>-9999</v>
@@ -7915,19 +8755,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7935,13 +8775,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>80</v>
@@ -7952,13 +8792,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>80</v>
@@ -7969,13 +8809,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>80</v>
@@ -7986,13 +8826,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>80</v>
@@ -8003,13 +8843,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>50</v>
@@ -8020,13 +8860,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>13</v>
@@ -8037,13 +8877,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>66</v>
+        <v>97</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>30</v>
@@ -8054,13 +8894,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>50</v>
@@ -8071,13 +8911,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>13</v>
@@ -8088,13 +8928,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>120</v>
@@ -8105,13 +8945,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -8122,13 +8962,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>80</v>
@@ -8139,13 +8979,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>999</v>
@@ -8156,13 +8996,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>999</v>
@@ -8173,13 +9013,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>999</v>
@@ -8190,13 +9030,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>999</v>
@@ -8207,13 +9047,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>999</v>
@@ -8224,13 +9064,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>999</v>
@@ -8241,13 +9081,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>999</v>
@@ -8258,13 +9098,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>999</v>
@@ -8275,13 +9115,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>999</v>
@@ -8292,13 +9132,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>999</v>
@@ -8328,70 +9168,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>115</v>
+        <v>146</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>119</v>
+        <v>150</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
@@ -9250,70 +10090,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>115</v>
+        <v>146</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>119</v>
+        <v>150</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>120</v>
+        <v>151</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9353,34 +10193,34 @@
       <c r="L2" s="2" t="n">
         <v>1.26813</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="M2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="P2" s="4" t="n">
+      <c r="P2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="Q2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="R2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="S2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="T2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="U2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V2" s="1" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9421,34 +10261,34 @@
       <c r="L3" s="2" t="n">
         <v>-0.21981</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="M3" s="1" t="n">
         <v>1.201</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N3" s="1" t="n">
         <v>1.401</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="O3" s="1" t="n">
         <v>1.75</v>
       </c>
-      <c r="P3" s="4" t="n">
+      <c r="P3" s="1" t="n">
         <v>1.106</v>
       </c>
-      <c r="Q3" s="4" t="n">
+      <c r="Q3" s="1" t="n">
         <v>0.432</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="R3" s="1" t="n">
         <v>-0.04</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="S3" s="1" t="n">
         <v>0.348</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="T3" s="1" t="n">
         <v>-0.328</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="U3" s="1" t="n">
         <v>-0.328</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="V3" s="1" t="n">
         <v>-0.428</v>
       </c>
     </row>
@@ -9489,34 +10329,34 @@
       <c r="L4" s="2" t="n">
         <v>-0.1405</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="1" t="n">
         <v>0.391</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="1" t="n">
         <v>0.476</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="1" t="n">
         <v>0.321</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="1" t="n">
         <v>0.421</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="1" t="n">
         <v>0.426</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="1" t="n">
         <v>0.708</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="1" t="n">
         <v>0.326</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="1" t="n">
         <v>0.64</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U4" s="1" t="n">
         <v>0.64</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="V4" s="1" t="n">
         <v>0.667</v>
       </c>
     </row>
@@ -9627,4 +10467,573 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultColWidth="12.8046875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="n">
+        <v>0.072</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="n">
+        <v>1.371</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1.491</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.943</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="n">
+        <v>1.402</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>1.349</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="n">
+        <v>0.002697</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.001491</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1" t="n">
+        <v>0.000596</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.000642</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="n">
+        <v>9.86E-005</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.000207</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="4" t="n">
+        <v>3.27E-006</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1.34E-005</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="4" t="n">
+        <v>1.08E-006</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>8.63E-006</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="4" t="n">
+        <v>3.58E-007</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>5.57E-006</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="4" t="n">
+        <v>1.19E-007</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>3.6E-006</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>2.32E-006</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>1.5E-006</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>9.68E-007</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>2.61E-007</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>1.16E-007</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add PRELES multiple species (select the most abundant to run)
</commit_message>
<xml_diff>
--- a/data/PREBAS_parameters.xlsx
+++ b/data/PREBAS_parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="pPRELES" sheetId="1" state="visible" r:id="rId3"/>
@@ -16,6 +16,7 @@
     <sheet name="pAWEN" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="pHcM" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="pPeattp" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="pPRELES_matrix" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -39,7 +40,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -66,7 +66,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -81,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="246">
   <si>
     <t xml:space="preserve">pPRELESnames</t>
   </si>
@@ -856,7 +855,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -907,7 +905,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -926,6 +924,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3089,7 +3091,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W54"/>
+  <dimension ref="A1:AH59"/>
   <sheetFormatPr defaultColWidth="8.3828125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="22.36"/>
@@ -6929,6 +6931,71 @@
       <c r="W54" s="1" t="n">
         <v>-9999</v>
       </c>
+    </row>
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X55" s="1"/>
+      <c r="Y55" s="1"/>
+      <c r="Z55" s="1"/>
+      <c r="AA55" s="1"/>
+      <c r="AB55" s="1"/>
+      <c r="AC55" s="1"/>
+      <c r="AD55" s="1"/>
+      <c r="AE55" s="1"/>
+      <c r="AF55" s="1"/>
+      <c r="AG55" s="1"/>
+      <c r="AH55" s="1"/>
+    </row>
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X56" s="1"/>
+      <c r="Y56" s="1"/>
+      <c r="Z56" s="1"/>
+      <c r="AA56" s="1"/>
+      <c r="AB56" s="1"/>
+      <c r="AC56" s="1"/>
+      <c r="AD56" s="1"/>
+      <c r="AE56" s="1"/>
+      <c r="AF56" s="1"/>
+      <c r="AG56" s="1"/>
+      <c r="AH56" s="1"/>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X57" s="1"/>
+      <c r="Y57" s="1"/>
+      <c r="Z57" s="1"/>
+      <c r="AA57" s="1"/>
+      <c r="AB57" s="1"/>
+      <c r="AC57" s="1"/>
+      <c r="AD57" s="1"/>
+      <c r="AE57" s="1"/>
+      <c r="AF57" s="1"/>
+      <c r="AG57" s="1"/>
+      <c r="AH57" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X58" s="1"/>
+      <c r="Y58" s="1"/>
+      <c r="Z58" s="1"/>
+      <c r="AA58" s="1"/>
+      <c r="AB58" s="1"/>
+      <c r="AC58" s="1"/>
+      <c r="AD58" s="1"/>
+      <c r="AE58" s="1"/>
+      <c r="AF58" s="1"/>
+      <c r="AG58" s="1"/>
+      <c r="AH58" s="1"/>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X59" s="1"/>
+      <c r="Y59" s="1"/>
+      <c r="Z59" s="1"/>
+      <c r="AA59" s="1"/>
+      <c r="AB59" s="1"/>
+      <c r="AC59" s="1"/>
+      <c r="AD59" s="1"/>
+      <c r="AE59" s="1"/>
+      <c r="AF59" s="1"/>
+      <c r="AG59" s="1"/>
+      <c r="AH59" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -11036,4 +11103,2864 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:W41"/>
+  <sheetFormatPr defaultColWidth="12.8046875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>614.544134</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="P2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="R2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="S2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="T2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="V2" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="W2" s="5" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>0.118</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>1.312411455</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="M6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="N6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="P6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="R6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="S6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="T6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="U6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="V6" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="W6" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="S7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="W7" s="1" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="M10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="N10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="P10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="R10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="S10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="T10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="U10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="V10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="W10" s="1" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="M11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="P11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="R11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="S11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="T11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="U11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V11" s="1" t="n">
+        <v>2000</v>
+      </c>
+      <c r="W11" s="1" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0.7457</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0.7457</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0.7457</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1.004588094</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0.820124449</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="V12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+      <c r="W12" s="2" t="n">
+        <v>0.748464</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>2.187171797</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>5.650375927</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="V13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>12.74915</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>-3.063</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>-3.063</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>-3.063</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>-9.937886741</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>-3.19169985</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="V14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+      <c r="W14" s="2" t="n">
+        <v>-3.566967</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>23.33402032</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>17.45828968</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="V15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+      <c r="W15" s="2" t="n">
+        <v>18.4513</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>-0.1027</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>-0.1027</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>-0.1027</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>-0.078699766</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>-0.158842341</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="O16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="R16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="S16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="T16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="U16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="V16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+      <c r="W16" s="5" t="n">
+        <v>-0.136732</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.03673</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>0.03673</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0.03673</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.05678157</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0.033324665</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="V17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>0.033942</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>0.7779</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>0.7779</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>0.7779</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.43569651</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0.650491581</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="V18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+      <c r="W18" s="2" t="n">
+        <v>0.448975</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W19" s="2" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="V20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+      <c r="W20" s="2" t="n">
+        <v>-0.364</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="V21" s="2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="W21" s="2" t="n">
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>0.2715</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>0.2715</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>0.2715</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0.216867322</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>0.119428078</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="R22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="V22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+      <c r="W22" s="2" t="n">
+        <v>0.33271</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>0.8351</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0.8351</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>0.8351</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.886165542</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>0.899640533</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="V23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+      <c r="W23" s="2" t="n">
+        <v>0.857291</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0.07348</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0.07348</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0.07348</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0.076537373</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0.163152905</v>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="M24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="N24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="O24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="P24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="Q24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="R24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="S24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="T24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="U24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="V24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+      <c r="W24" s="5" t="n">
+        <v>0.041781</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>0.9996</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0.9996</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0.9996</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0.250944646</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>0.999200597</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="V25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+      <c r="W25" s="2" t="n">
+        <v>0.474173</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>0.4428</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0.4428</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0.4428</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>2.484834199</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>0.623269245</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="V26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+      <c r="W26" s="2" t="n">
+        <v>0.278332</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="W27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="V28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="W28" s="2" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>4.970496</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>4.970496</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>4.970496</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0.992544622</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>4.35800751</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="V29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+      <c r="W29" s="2" t="n">
+        <v>4.824704</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="V32" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="W32" s="2" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>-7.9532</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="J36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="N36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="O36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="P36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="R36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="S36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="T36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="U36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="V36" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="W36" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="F37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="I37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="J37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="M37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="N37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="O37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="P37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="R37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="S37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="T37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="U37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="V37" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="W37" s="1" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="T38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="U38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="V38" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="W38" s="2" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="U39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="V39" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="W39" s="2" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>-999</v>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="M40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="N40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="O40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="P40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="Q40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="R40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="S40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="T40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="U40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="V40" s="5" t="n">
+        <v>-999</v>
+      </c>
+      <c r="W40" s="5" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update CO2model parameters (again)
</commit_message>
<xml_diff>
--- a/data/PREBAS_parameters.xlsx
+++ b/data/PREBAS_parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="pPRELES" sheetId="1" state="visible" r:id="rId3"/>
@@ -1086,7 +1086,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1107,7 +1107,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1117,10 +1117,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -18484,13 +18480,13 @@
       <c r="W2" s="6" t="n">
         <v>413</v>
       </c>
-      <c r="X2" s="8" t="n">
+      <c r="X2" s="5" t="n">
         <v>1396.067</v>
       </c>
-      <c r="Y2" s="8" t="n">
+      <c r="Y2" s="5" t="n">
         <v>971.32524921</v>
       </c>
-      <c r="Z2" s="9" t="n">
+      <c r="Z2" s="8" t="n">
         <v>1917.6</v>
       </c>
     </row>
@@ -18564,7 +18560,7 @@
       <c r="W3" s="6" t="n">
         <v>0.45</v>
       </c>
-      <c r="X3" s="8" t="n">
+      <c r="X3" s="5" t="n">
         <v>0.358</v>
       </c>
       <c r="Y3" s="6" t="n">
@@ -18644,7 +18640,7 @@
       <c r="W4" s="6" t="n">
         <v>0.118</v>
       </c>
-      <c r="X4" s="8" t="n">
+      <c r="X4" s="5" t="n">
         <v>0.156</v>
       </c>
       <c r="Y4" s="6" t="n">
@@ -18724,7 +18720,7 @@
       <c r="W5" s="6" t="n">
         <v>1.00156207438108</v>
       </c>
-      <c r="X5" s="8" t="n">
+      <c r="X5" s="5" t="n">
         <v>2.13588811</v>
       </c>
       <c r="Y5" s="6" t="n">
@@ -18804,7 +18800,7 @@
       <c r="W6" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="X6" s="8" t="n">
+      <c r="X6" s="5" t="n">
         <v>0.8</v>
       </c>
       <c r="Y6" s="6" t="n">
@@ -18884,7 +18880,7 @@
       <c r="W7" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="X7" s="8" t="n">
+      <c r="X7" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y7" s="6" t="n">
@@ -18964,7 +18960,7 @@
       <c r="W8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="X8" s="8" t="n">
+      <c r="X8" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y8" s="6" t="n">
@@ -19044,7 +19040,7 @@
       <c r="W9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="X9" s="8" t="n">
+      <c r="X9" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y9" s="6" t="n">
@@ -19124,7 +19120,7 @@
       <c r="W10" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="X10" s="8" t="n">
+      <c r="X10" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y10" s="6" t="n">
@@ -19204,7 +19200,7 @@
       <c r="W11" s="6" t="n">
         <v>2000</v>
       </c>
-      <c r="X11" s="8" t="n">
+      <c r="X11" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y11" s="6" t="n">
@@ -19284,13 +19280,13 @@
       <c r="W12" s="6" t="n">
         <v>0.711245310135586</v>
       </c>
-      <c r="X12" s="10" t="n">
+      <c r="X12" s="9" t="n">
         <v>0.9998057</v>
       </c>
-      <c r="Y12" s="8" t="n">
+      <c r="Y12" s="5" t="n">
         <v>0.78045355</v>
       </c>
-      <c r="Z12" s="11" t="n">
+      <c r="Z12" s="10" t="n">
         <v>1.097058</v>
       </c>
     </row>
@@ -19364,13 +19360,13 @@
       <c r="W13" s="6" t="n">
         <v>2.48358288498399</v>
       </c>
-      <c r="X13" s="10" t="n">
+      <c r="X13" s="9" t="n">
         <v>13.0225</v>
       </c>
-      <c r="Y13" s="8" t="n">
+      <c r="Y13" s="5" t="n">
         <v>7.0079237</v>
       </c>
-      <c r="Z13" s="11" t="n">
+      <c r="Z13" s="10" t="n">
         <v>14.98661</v>
       </c>
     </row>
@@ -19444,13 +19440,13 @@
       <c r="W14" s="6" t="n">
         <v>-6.01042831420331</v>
       </c>
-      <c r="X14" s="10" t="n">
+      <c r="X14" s="9" t="n">
         <v>5.71606</v>
       </c>
-      <c r="Y14" s="8" t="n">
+      <c r="Y14" s="5" t="n">
         <v>-4.37275471</v>
       </c>
-      <c r="Z14" s="11" t="n">
+      <c r="Z14" s="10" t="n">
         <v>4.839464</v>
       </c>
     </row>
@@ -19524,13 +19520,13 @@
       <c r="W15" s="6" t="n">
         <v>17.2734188291157</v>
       </c>
-      <c r="X15" s="10" t="n">
+      <c r="X15" s="9" t="n">
         <v>13.03214</v>
       </c>
-      <c r="Y15" s="8" t="n">
+      <c r="Y15" s="5" t="n">
         <v>15.00670035</v>
       </c>
-      <c r="Z15" s="11" t="n">
+      <c r="Z15" s="10" t="n">
         <v>16.69706</v>
       </c>
     </row>
@@ -19604,13 +19600,13 @@
       <c r="W16" s="6" t="n">
         <v>-0.0188432127763177</v>
       </c>
-      <c r="X16" s="10" t="n">
+      <c r="X16" s="9" t="n">
         <v>-0.2879784</v>
       </c>
-      <c r="Y16" s="8" t="n">
+      <c r="Y16" s="5" t="n">
         <v>-0.34870743</v>
       </c>
-      <c r="Z16" s="11" t="n">
+      <c r="Z16" s="10" t="n">
         <v>-0.1069248</v>
       </c>
     </row>
@@ -19684,13 +19680,13 @@
       <c r="W17" s="6" t="n">
         <v>0.0581182268266003</v>
       </c>
-      <c r="X17" s="10" t="n">
+      <c r="X17" s="9" t="n">
         <v>0.04019984</v>
       </c>
-      <c r="Y17" s="8" t="n">
+      <c r="Y17" s="5" t="n">
         <v>0.02813683</v>
       </c>
-      <c r="Z17" s="11" t="n">
+      <c r="Z17" s="10" t="n">
         <v>0.02578476</v>
       </c>
     </row>
@@ -19764,13 +19760,13 @@
       <c r="W18" s="6" t="n">
         <v>0.543125003489455</v>
       </c>
-      <c r="X18" s="10" t="n">
+      <c r="X18" s="9" t="n">
         <v>0.0002527681</v>
       </c>
-      <c r="Y18" s="8" t="n">
+      <c r="Y18" s="5" t="n">
         <v>0.99895546</v>
       </c>
-      <c r="Z18" s="11" t="n">
+      <c r="Z18" s="10" t="n">
         <v>0.9972443</v>
       </c>
     </row>
@@ -19778,79 +19774,79 @@
       <c r="A19" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="F19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="G19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="H19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="I19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="K19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="M19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="N19" s="12" t="n">
-        <v>-0.364</v>
-      </c>
-      <c r="O19" s="12" t="n">
+      <c r="B19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="P19" s="12" t="n">
+      <c r="C19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="Q19" s="12" t="n">
+      <c r="D19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="R19" s="12" t="n">
+      <c r="E19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="S19" s="12" t="n">
+      <c r="F19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="T19" s="12" t="n">
+      <c r="G19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="U19" s="12" t="n">
+      <c r="H19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="V19" s="12" t="n">
+      <c r="I19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="W19" s="12" t="n">
+      <c r="J19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="X19" s="12" t="n">
+      <c r="K19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="Y19" s="12" t="n">
+      <c r="L19" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="Z19" s="12" t="n">
+      <c r="M19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="O19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="P19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="R19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="S19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="T19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="U19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="W19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="X19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y19" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Z19" s="11" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -20004,7 +20000,7 @@
       <c r="W21" s="6" t="n">
         <v>-15</v>
       </c>
-      <c r="X21" s="8" t="n">
+      <c r="X21" s="5" t="n">
         <v>-999</v>
       </c>
       <c r="Y21" s="6" t="n">
@@ -20084,13 +20080,13 @@
       <c r="W22" s="6" t="n">
         <v>0.278328809531619</v>
       </c>
-      <c r="X22" s="10" t="n">
+      <c r="X22" s="9" t="n">
         <v>0.2229754</v>
       </c>
-      <c r="Y22" s="8" t="n">
+      <c r="Y22" s="5" t="n">
         <v>0.17896756</v>
       </c>
-      <c r="Z22" s="11" t="n">
+      <c r="Z22" s="10" t="n">
         <v>0.2733934</v>
       </c>
     </row>
@@ -20164,13 +20160,13 @@
       <c r="W23" s="6" t="n">
         <v>0.477158761193225</v>
       </c>
-      <c r="X23" s="10" t="n">
+      <c r="X23" s="9" t="n">
         <v>0.9998016</v>
       </c>
-      <c r="Y23" s="8" t="n">
+      <c r="Y23" s="5" t="n">
         <v>0.83457793</v>
       </c>
-      <c r="Z23" s="11" t="n">
+      <c r="Z23" s="10" t="n">
         <v>0.9322595</v>
       </c>
     </row>
@@ -20244,13 +20240,13 @@
       <c r="W24" s="6" t="n">
         <v>0.0733362748652165</v>
       </c>
-      <c r="X24" s="10" t="n">
+      <c r="X24" s="9" t="n">
         <v>0.1196433</v>
       </c>
-      <c r="Y24" s="8" t="n">
+      <c r="Y24" s="5" t="n">
         <v>0.23431144</v>
       </c>
-      <c r="Z24" s="11" t="n">
+      <c r="Z24" s="10" t="n">
         <v>0.09425691</v>
       </c>
     </row>
@@ -20324,13 +20320,13 @@
       <c r="W25" s="6" t="n">
         <v>0.760231646290861</v>
       </c>
-      <c r="X25" s="10" t="n">
+      <c r="X25" s="9" t="n">
         <v>0.9995386</v>
       </c>
-      <c r="Y25" s="8" t="n">
+      <c r="Y25" s="5" t="n">
         <v>0.41021161</v>
       </c>
-      <c r="Z25" s="11" t="n">
+      <c r="Z25" s="10" t="n">
         <v>0.9968247</v>
       </c>
     </row>
@@ -20404,13 +20400,13 @@
       <c r="W26" s="6" t="n">
         <v>0.473671920042078</v>
       </c>
-      <c r="X26" s="10" t="n">
+      <c r="X26" s="9" t="n">
         <v>1.266691</v>
       </c>
-      <c r="Y26" s="8" t="n">
+      <c r="Y26" s="5" t="n">
         <v>1.27262003</v>
       </c>
-      <c r="Z26" s="11" t="n">
+      <c r="Z26" s="10" t="n">
         <v>0.0002090931</v>
       </c>
     </row>
@@ -20484,7 +20480,7 @@
       <c r="W27" s="6" t="n">
         <v>1.2</v>
       </c>
-      <c r="X27" s="8" t="n">
+      <c r="X27" s="5" t="n">
         <v>1.2</v>
       </c>
       <c r="Y27" s="6" t="n">
@@ -20564,7 +20560,7 @@
       <c r="W28" s="6" t="n">
         <v>0.33</v>
       </c>
-      <c r="X28" s="8" t="n">
+      <c r="X28" s="5" t="n">
         <v>0.33</v>
       </c>
       <c r="Y28" s="6" t="n">
@@ -20644,13 +20640,13 @@
       <c r="W29" s="6" t="n">
         <v>4.970496</v>
       </c>
-      <c r="X29" s="8" t="n">
+      <c r="X29" s="5" t="n">
         <v>5.20151518</v>
       </c>
-      <c r="Y29" s="8" t="n">
+      <c r="Y29" s="5" t="n">
         <v>1.22350796</v>
       </c>
-      <c r="Z29" s="11" t="n">
+      <c r="Z29" s="10" t="n">
         <v>1.758379</v>
       </c>
     </row>
@@ -20724,7 +20720,7 @@
       <c r="W30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="X30" s="8" t="n">
+      <c r="X30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Y30" s="6" t="n">
@@ -20804,7 +20800,7 @@
       <c r="W31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="X31" s="8" t="n">
+      <c r="X31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Y31" s="6" t="n">
@@ -20884,7 +20880,7 @@
       <c r="W32" s="6" t="n">
         <v>160</v>
       </c>
-      <c r="X32" s="8" t="n">
+      <c r="X32" s="5" t="n">
         <v>200</v>
       </c>
       <c r="Y32" s="6" t="n">
@@ -20964,7 +20960,7 @@
       <c r="W33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="X33" s="8" t="n">
+      <c r="X33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Y33" s="6" t="n">

</xml_diff>